<commit_message>
Auto update Balance Pick Summary
</commit_message>
<xml_diff>
--- a/Balance_Pick_Summary.xlsx
+++ b/Balance_Pick_Summary.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="22">
   <si>
     <t>WAVE_NBR</t>
   </si>
@@ -80,13 +80,7 @@
     <t>SP-HLIN</t>
   </si>
   <si>
-    <t>SP-HMEN</t>
-  </si>
-  <si>
     <t>SP-HWNTR</t>
-  </si>
-  <si>
-    <t>SP-PERFUME</t>
   </si>
   <si>
     <t>SPAIS1</t>
@@ -648,11 +642,11 @@
         <v>21090</v>
       </c>
       <c r="C11" s="3">
-        <v>196</v>
+        <v>166</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3">
-        <v>196</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -661,13 +655,13 @@
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="4">
-        <v>196</v>
+        <v>166</v>
       </c>
       <c r="D12" s="4">
         <v>23</v>
       </c>
       <c r="E12" s="4">
-        <v>219</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -878,10 +872,10 @@
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3">
-        <v>376</v>
+        <v>353</v>
       </c>
       <c r="L8" s="3">
-        <v>376</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -900,10 +894,10 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="L9" s="3">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -922,10 +916,10 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="L10" s="3">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -936,7 +930,7 @@
         <v>60127</v>
       </c>
       <c r="C11" s="3">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3">
@@ -949,7 +943,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -960,11 +954,9 @@
         <v>60132</v>
       </c>
       <c r="C12" s="3">
-        <v>115</v>
-      </c>
-      <c r="D12" s="3">
-        <v>1</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="D12" s="3"/>
       <c r="E12" s="3">
         <v>1</v>
       </c>
@@ -975,7 +967,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3">
-        <v>117</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -986,7 +978,7 @@
         <v>60139</v>
       </c>
       <c r="C13" s="3">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3">
@@ -999,7 +991,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1254,10 +1246,10 @@
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
       <c r="K24" s="3">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="L24" s="3">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1280,10 +1272,10 @@
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3">
-        <v>453</v>
+        <v>443</v>
       </c>
       <c r="L25" s="3">
-        <v>493</v>
+        <v>483</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1304,10 +1296,10 @@
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
       <c r="K26" s="3">
-        <v>499</v>
+        <v>489</v>
       </c>
       <c r="L26" s="3">
-        <v>521</v>
+        <v>511</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1373,7 +1365,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I29" s="3">
         <v>2</v>
@@ -1381,7 +1373,7 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1399,7 +1391,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="I30" s="3">
         <v>1</v>
@@ -1407,7 +1399,7 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3">
-        <v>114</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1425,13 +1417,13 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1449,13 +1441,13 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1471,13 +1463,13 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1495,13 +1487,13 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1517,13 +1509,13 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3">
-        <v>232</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1608,12 +1600,12 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3">
-        <v>284</v>
+        <v>280</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -1630,12 +1622,12 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -1652,12 +1644,12 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -1674,12 +1666,12 @@
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -1696,12 +1688,12 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
       <c r="L43" s="3">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -1718,12 +1710,12 @@
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
       <c r="I44" s="3">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
       <c r="L44" s="3">
-        <v>215</v>
+        <v>198</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2234,10 +2226,10 @@
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="4">
-        <v>1146</v>
+        <v>1129</v>
       </c>
       <c r="D67" s="4">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E67" s="4">
         <v>16</v>
@@ -2249,19 +2241,19 @@
         <v>2723</v>
       </c>
       <c r="H67" s="4">
-        <v>960</v>
+        <v>916</v>
       </c>
       <c r="I67" s="4">
-        <v>1123</v>
+        <v>1094</v>
       </c>
       <c r="J67" s="4">
         <v>98</v>
       </c>
       <c r="K67" s="4">
-        <v>2111</v>
+        <v>2052</v>
       </c>
       <c r="L67" s="4">
-        <v>9033</v>
+        <v>8883</v>
       </c>
     </row>
   </sheetData>
@@ -2309,10 +2301,10 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2325,10 +2317,10 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F3" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2340,11 +2332,11 @@
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2356,11 +2348,11 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2404,13 +2396,13 @@
         <v>14</v>
       </c>
       <c r="D8" s="4">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="E8" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F8" s="4">
-        <v>75</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2476,18 +2468,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="5" width="9.7109375" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="8.7109375" customWidth="1"/>
-    <col min="9" max="9" width="7.7109375" customWidth="1"/>
+    <col min="2" max="4" width="9.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2507,16 +2498,10 @@
         <v>21</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:7">
       <c r="A2" s="2">
         <v>3004</v>
       </c>
@@ -2524,24 +2509,20 @@
         <v>21082</v>
       </c>
       <c r="C2" s="3">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D2" s="3">
         <v>21</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3">
+        <v>70</v>
+      </c>
       <c r="G2" s="3">
-        <v>2</v>
-      </c>
-      <c r="H2" s="3">
-        <v>78</v>
-      </c>
-      <c r="I2" s="3">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="2">
         <v>3004</v>
       </c>
@@ -2549,24 +2530,20 @@
         <v>21234</v>
       </c>
       <c r="C3" s="3">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D3" s="3">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="F3" s="3">
+        <v>55</v>
+      </c>
       <c r="G3" s="3">
-        <v>1</v>
-      </c>
-      <c r="H3" s="3">
-        <v>59</v>
-      </c>
-      <c r="I3" s="3">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="2">
         <v>3006</v>
       </c>
@@ -2580,20 +2557,16 @@
         <v>23</v>
       </c>
       <c r="E4" s="3">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F4" s="3">
-        <v>32</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
         <v>14</v>
       </c>
-      <c r="I4" s="3">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="G4" s="3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="2">
         <v>3006</v>
       </c>
@@ -2607,44 +2580,34 @@
         <v>20</v>
       </c>
       <c r="E5" s="3">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="F5" s="3">
-        <v>21</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3">
         <v>4</v>
       </c>
-      <c r="I5" s="3">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="G5" s="3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="4">
-        <v>181</v>
+        <v>156</v>
       </c>
       <c r="D6" s="4">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E6" s="4">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F6" s="4">
-        <v>53</v>
+        <v>143</v>
       </c>
       <c r="G6" s="4">
-        <v>3</v>
-      </c>
-      <c r="H6" s="4">
-        <v>155</v>
-      </c>
-      <c r="I6" s="4">
-        <v>529</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>